<commit_message>
Before change the whole augmentation
</commit_message>
<xml_diff>
--- a/labeled/Add_Eating/July/sip_volume_distribution_after_augmentation.xlsx
+++ b/labeled/Add_Eating/July/sip_volume_distribution_after_augmentation.xlsx
@@ -455,7 +455,7 @@
         <v>2.5</v>
       </c>
       <c r="C2" t="n">
-        <v>44</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3">
@@ -468,7 +468,7 @@
         <v>7.5</v>
       </c>
       <c r="C3" t="n">
-        <v>40</v>
+        <v>440</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +481,7 @@
         <v>12.5</v>
       </c>
       <c r="C4" t="n">
-        <v>80</v>
+        <v>880</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         <v>17.5</v>
       </c>
       <c r="C5" t="n">
-        <v>74</v>
+        <v>814</v>
       </c>
     </row>
     <row r="6">
@@ -507,7 +507,7 @@
         <v>22.5</v>
       </c>
       <c r="C6" t="n">
-        <v>85</v>
+        <v>935</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         <v>27.5</v>
       </c>
       <c r="C7" t="n">
-        <v>981</v>
+        <v>599</v>
       </c>
     </row>
     <row r="8">
@@ -533,7 +533,7 @@
         <v>32.5</v>
       </c>
       <c r="C8" t="n">
-        <v>620</v>
+        <v>372</v>
       </c>
     </row>
     <row r="9">
@@ -546,7 +546,7 @@
         <v>37.5</v>
       </c>
       <c r="C9" t="n">
-        <v>700</v>
+        <v>420</v>
       </c>
     </row>
     <row r="10">
@@ -559,7 +559,7 @@
         <v>42.5</v>
       </c>
       <c r="C10" t="n">
-        <v>664</v>
+        <v>432</v>
       </c>
     </row>
     <row r="11">
@@ -572,7 +572,7 @@
         <v>47.5</v>
       </c>
       <c r="C11" t="n">
-        <v>285</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12">
@@ -585,7 +585,7 @@
         <v>52.5</v>
       </c>
       <c r="C12" t="n">
-        <v>290</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13">
@@ -598,7 +598,7 @@
         <v>57.5</v>
       </c>
       <c r="C13" t="n">
-        <v>600</v>
+        <v>400</v>
       </c>
     </row>
     <row r="14">
@@ -611,7 +611,7 @@
         <v>62.5</v>
       </c>
       <c r="C14" t="n">
-        <v>384</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15">
@@ -624,7 +624,7 @@
         <v>67.5</v>
       </c>
       <c r="C15" t="n">
-        <v>186</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16">
@@ -637,7 +637,7 @@
         <v>72.5</v>
       </c>
       <c r="C16" t="n">
-        <v>186</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17">
@@ -650,7 +650,7 @@
         <v>77.5</v>
       </c>
       <c r="C17" t="n">
-        <v>336</v>
+        <v>224</v>
       </c>
     </row>
     <row r="18">
@@ -663,7 +663,7 @@
         <v>82.5</v>
       </c>
       <c r="C18" t="n">
-        <v>230</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19">
@@ -676,7 +676,7 @@
         <v>87.5</v>
       </c>
       <c r="C19" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20">
@@ -689,7 +689,7 @@
         <v>92.5</v>
       </c>
       <c r="C20" t="n">
-        <v>120</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21">
@@ -702,7 +702,7 @@
         <v>97.5</v>
       </c>
       <c r="C21" t="n">
-        <v>288</v>
+        <v>192</v>
       </c>
     </row>
     <row r="22">
@@ -715,7 +715,7 @@
         <v>102.5</v>
       </c>
       <c r="C22" t="n">
-        <v>192</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23">
@@ -767,7 +767,7 @@
         <v>122.5</v>
       </c>
       <c r="C26" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27">
@@ -780,7 +780,7 @@
         <v>127.5</v>
       </c>
       <c r="C27" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="28">
@@ -793,7 +793,7 @@
         <v>132.5</v>
       </c>
       <c r="C28" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="29">
@@ -819,7 +819,7 @@
         <v>142.5</v>
       </c>
       <c r="C30" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="31">
@@ -871,7 +871,7 @@
         <v>162.5</v>
       </c>
       <c r="C34" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>